<commit_message>
Finalize Superstore BI project deliverables
</commit_message>
<xml_diff>
--- a/Excel/Superstore.xlsx
+++ b/Excel/Superstore.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI project\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08DFF524-EF18-46DB-82A8-4B4DB9E08A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FC9A0D-8C78-4593-BD80-E4A33B80AAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{22E721EE-254E-41D6-B265-106E2BD28AD9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{22E721EE-254E-41D6-B265-106E2BD28AD9}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot_Category_Region" sheetId="2" r:id="rId1"/>
@@ -20,10 +20,10 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
-    <pivotCache cacheId="1" r:id="rId6"/>
-    <pivotCache cacheId="2" r:id="rId7"/>
-    <pivotCache cacheId="16" r:id="rId8"/>
+    <pivotCache cacheId="30" r:id="rId5"/>
+    <pivotCache cacheId="33" r:id="rId6"/>
+    <pivotCache cacheId="36" r:id="rId7"/>
+    <pivotCache cacheId="39" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -4967,7 +4967,339 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46181.646085185188" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{16152C29-77A8-44C6-B6A6-9557FF558682}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46206.740127314813" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{8648899E-E912-41E9-AC6C-35175A7D3FBA}">
+  <cacheSource type="external" connectionId="2"/>
+  <cacheFields count="2">
+    <cacheField name="[Dim Product].[Category].[Category]" caption="Category" numFmtId="0" hierarchy="10" level="1">
+      <sharedItems count="3">
+        <s v="[Dim Product].[Category].&amp;[Furniture]" c="Furniture"/>
+        <s v="[Dim Product].[Category].&amp;[Office Supplies]" c="Office Supplies"/>
+        <s v="[Dim Product].[Category].&amp;[Technology]" c="Technology"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[Profit Margin]" caption="Profit Margin" numFmtId="0" hierarchy="38" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="40">
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer]" caption="Customer" defaultMemberUniqueName="[Dim Customer].[Customer].[All]" allUniqueName="[Dim Customer].[Customer].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[Dim Customer].[Customer ID].[All]" allUniqueName="[Dim Customer].[Customer ID].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer Name]" caption="Customer Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Customer].[Customer Name].[All]" allUniqueName="[Dim Customer].[Customer Name].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Dim Customer].[Segment].[All]" allUniqueName="[Dim Customer].[Segment].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[City]" caption="City" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Geography].[City].[All]" allUniqueName="[Dim Geography].[City].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Dim Geography].[Country].[All]" allUniqueName="[Dim Geography].[Country].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Geography]" caption="Geography" defaultMemberUniqueName="[Dim Geography].[Geography].[All]" allUniqueName="[Dim Geography].[Geography].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Postal Code]" caption="Postal Code" attribute="1" defaultMemberUniqueName="[Dim Geography].[Postal Code].[All]" allUniqueName="[Dim Geography].[Postal Code].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Region]" caption="Region" attribute="1" defaultMemberUniqueName="[Dim Geography].[Region].[All]" allUniqueName="[Dim Geography].[Region].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[State]" caption="State" attribute="1" defaultMemberUniqueName="[Dim Geography].[State].[All]" allUniqueName="[Dim Geography].[State].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Category].[All]" allUniqueName="[Dim Product].[Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="2" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Dim Product].[Product]" caption="Product" defaultMemberUniqueName="[Dim Product].[Product].[All]" allUniqueName="[Dim Product].[Product].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product ID]" caption="Product ID" attribute="1" defaultMemberUniqueName="[Dim Product].[Product ID].[All]" allUniqueName="[Dim Product].[Product ID].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product Name]" caption="Product Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Product].[Product Name].[All]" allUniqueName="[Dim Product].[Product Name].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Sub Category]" caption="Sub Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Sub Category].[All]" allUniqueName="[Dim Product].[Sub Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Ship Mode].[Ship Mode]" caption="Ship Mode" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Ship Mode].[Ship Mode].[All]" allUniqueName="[Dim Ship Mode].[Ship Mode].[All]" dimensionUniqueName="[Dim Ship Mode]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Calendar]" caption="Order Date.Calendar" defaultMemberUniqueName="[Order Date].[Calendar].[All]" allUniqueName="[Order Date].[Calendar].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Day]" caption="Order Date.Day" attribute="1" defaultMemberUniqueName="[Order Date].[Day].[All]" allUniqueName="[Order Date].[Day].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Full Date]" caption="Order Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Order Date].[Full Date].[All]" allUniqueName="[Order Date].[Full Date].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Month]" caption="Order Date.Month" attribute="1" defaultMemberUniqueName="[Order Date].[Month].[All]" allUniqueName="[Order Date].[Month].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Month Name]" caption="Order Date.Month Name" attribute="1" defaultMemberUniqueName="[Order Date].[Month Name].[All]" allUniqueName="[Order Date].[Month Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Quarter]" caption="Order Date.Quarter" attribute="1" defaultMemberUniqueName="[Order Date].[Quarter].[All]" allUniqueName="[Order Date].[Quarter].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Weekday Name]" caption="Order Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Order Date].[Weekday Name].[All]" allUniqueName="[Order Date].[Weekday Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Year]" caption="Order Date.Year" attribute="1" defaultMemberUniqueName="[Order Date].[Year].[All]" allUniqueName="[Order Date].[Year].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Calendar]" caption="Ship Date.Calendar" defaultMemberUniqueName="[Ship Date].[Calendar].[All]" allUniqueName="[Ship Date].[Calendar].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Day]" caption="Ship Date.Day" attribute="1" defaultMemberUniqueName="[Ship Date].[Day].[All]" allUniqueName="[Ship Date].[Day].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Full Date]" caption="Ship Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Ship Date].[Full Date].[All]" allUniqueName="[Ship Date].[Full Date].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Month]" caption="Ship Date.Month" attribute="1" defaultMemberUniqueName="[Ship Date].[Month].[All]" allUniqueName="[Ship Date].[Month].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Month Name]" caption="Ship Date.Month Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Month Name].[All]" allUniqueName="[Ship Date].[Month Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Quarter]" caption="Ship Date.Quarter" attribute="1" defaultMemberUniqueName="[Ship Date].[Quarter].[All]" allUniqueName="[Ship Date].[Quarter].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Weekday Name]" caption="Ship Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Weekday Name].[All]" allUniqueName="[Ship Date].[Weekday Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Year]" caption="Ship Date.Year" attribute="1" defaultMemberUniqueName="[Ship Date].[Year].[All]" allUniqueName="[Ship Date].[Year].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Sales]" caption="Sales" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Quantity]" caption="Quantity" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Discount]" caption="Discount" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Profit]" caption="Profit" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Delivery Days]" caption="Delivery Days" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Fact Sales Count]" caption="Fact Sales Count" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Profit Margin]" caption="Profit Margin" measure="1" displayFolder="" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Avg Delivery Days]" caption="Avg Delivery Days" measure="1" displayFolder="" count="0"/>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="7">
+    <dimension name="Dim Customer" uniqueName="[Dim Customer]" caption="Dim Customer"/>
+    <dimension name="Dim Geography" uniqueName="[Dim Geography]" caption="Dim Geography"/>
+    <dimension name="Dim Product" uniqueName="[Dim Product]" caption="Dim Product"/>
+    <dimension name="Dim Ship Mode" uniqueName="[Dim Ship Mode]" caption="Dim Ship Mode"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Order Date" uniqueName="[Order Date]" caption="Order Date"/>
+    <dimension name="Ship Date" uniqueName="[Ship Date]" caption="Ship Date"/>
+  </dimensions>
+  <measureGroups count="1">
+    <measureGroup name="Fact Sales" caption="Fact Sales"/>
+  </measureGroups>
+  <maps count="6">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="0" dimension="2"/>
+    <map measureGroup="0" dimension="3"/>
+    <map measureGroup="0" dimension="5"/>
+    <map measureGroup="0" dimension="6"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46206.740127893521" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{2B00A886-4FF8-4527-B1CA-9D438D508401}">
+  <cacheSource type="external" connectionId="1"/>
+  <cacheFields count="8">
+    <cacheField name="[Dim Product].[Product].[Category]" caption="Category" numFmtId="0" hierarchy="11" level="1">
+      <sharedItems count="3">
+        <s v="[Dim Product].[Product].[Category].&amp;[Furniture]" c="Furniture"/>
+        <s v="[Dim Product].[Product].[Category].&amp;[Office Supplies]" c="Office Supplies"/>
+        <s v="[Dim Product].[Product].[Category].&amp;[Technology]" c="Technology"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Dim Product].[Product].[Sub Category]" caption="Sub Category" numFmtId="0" hierarchy="11" level="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Dim Product].[Product].[Product Name]" caption="Product Name" numFmtId="0" hierarchy="11" level="3">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Dim Product].[Product].[Product Name].[Category]" caption="Category" propertyName="Category" numFmtId="0" hierarchy="11" level="3" memberPropertyField="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Dim Product].[Product].[Product Name].[Product ID]" caption="Product ID" propertyName="Product ID" numFmtId="0" hierarchy="11" level="3" memberPropertyField="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Dim Product].[Product].[Product Name].[Sub Category]" caption="Sub Category" propertyName="Sub Category" numFmtId="0" hierarchy="11" level="3" memberPropertyField="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Measures].[Sales]" caption="Sales" numFmtId="0" hierarchy="32" level="32767"/>
+    <cacheField name="[Dim Geography].[Region].[Region]" caption="Region" numFmtId="0" hierarchy="8" level="1">
+      <sharedItems count="4">
+        <s v="[Dim Geography].[Region].&amp;[Central]" c="Central"/>
+        <s v="[Dim Geography].[Region].&amp;[East]" c="East"/>
+        <s v="[Dim Geography].[Region].&amp;[South]" c="South"/>
+        <s v="[Dim Geography].[Region].&amp;[West]" c="West"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <cacheHierarchies count="40">
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer]" caption="Customer" defaultMemberUniqueName="[Dim Customer].[Customer].[All]" allUniqueName="[Dim Customer].[Customer].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[Dim Customer].[Customer ID].[All]" allUniqueName="[Dim Customer].[Customer ID].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer Name]" caption="Customer Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Customer].[Customer Name].[All]" allUniqueName="[Dim Customer].[Customer Name].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Dim Customer].[Segment].[All]" allUniqueName="[Dim Customer].[Segment].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[City]" caption="City" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Geography].[City].[All]" allUniqueName="[Dim Geography].[City].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Dim Geography].[Country].[All]" allUniqueName="[Dim Geography].[Country].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Geography]" caption="Geography" defaultMemberUniqueName="[Dim Geography].[Geography].[All]" allUniqueName="[Dim Geography].[Geography].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Postal Code]" caption="Postal Code" attribute="1" defaultMemberUniqueName="[Dim Geography].[Postal Code].[All]" allUniqueName="[Dim Geography].[Postal Code].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Region]" caption="Region" attribute="1" defaultMemberUniqueName="[Dim Geography].[Region].[All]" allUniqueName="[Dim Geography].[Region].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="2" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="7"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Dim Geography].[State]" caption="State" attribute="1" defaultMemberUniqueName="[Dim Geography].[State].[All]" allUniqueName="[Dim Geography].[State].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Category].[All]" allUniqueName="[Dim Product].[Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product]" caption="Product" defaultMemberUniqueName="[Dim Product].[Product].[All]" allUniqueName="[Dim Product].[Product].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="4" unbalanced="0">
+      <fieldsUsage count="4">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+        <fieldUsage x="1"/>
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Dim Product].[Product ID]" caption="Product ID" attribute="1" defaultMemberUniqueName="[Dim Product].[Product ID].[All]" allUniqueName="[Dim Product].[Product ID].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product Name]" caption="Product Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Product].[Product Name].[All]" allUniqueName="[Dim Product].[Product Name].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Sub Category]" caption="Sub Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Sub Category].[All]" allUniqueName="[Dim Product].[Sub Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Ship Mode].[Ship Mode]" caption="Ship Mode" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Ship Mode].[Ship Mode].[All]" allUniqueName="[Dim Ship Mode].[Ship Mode].[All]" dimensionUniqueName="[Dim Ship Mode]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Calendar]" caption="Order Date.Calendar" defaultMemberUniqueName="[Order Date].[Calendar].[All]" allUniqueName="[Order Date].[Calendar].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Day]" caption="Order Date.Day" attribute="1" defaultMemberUniqueName="[Order Date].[Day].[All]" allUniqueName="[Order Date].[Day].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Full Date]" caption="Order Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Order Date].[Full Date].[All]" allUniqueName="[Order Date].[Full Date].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Month]" caption="Order Date.Month" attribute="1" defaultMemberUniqueName="[Order Date].[Month].[All]" allUniqueName="[Order Date].[Month].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Month Name]" caption="Order Date.Month Name" attribute="1" defaultMemberUniqueName="[Order Date].[Month Name].[All]" allUniqueName="[Order Date].[Month Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Quarter]" caption="Order Date.Quarter" attribute="1" defaultMemberUniqueName="[Order Date].[Quarter].[All]" allUniqueName="[Order Date].[Quarter].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Weekday Name]" caption="Order Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Order Date].[Weekday Name].[All]" allUniqueName="[Order Date].[Weekday Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Year]" caption="Order Date.Year" attribute="1" defaultMemberUniqueName="[Order Date].[Year].[All]" allUniqueName="[Order Date].[Year].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Calendar]" caption="Ship Date.Calendar" defaultMemberUniqueName="[Ship Date].[Calendar].[All]" allUniqueName="[Ship Date].[Calendar].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Day]" caption="Ship Date.Day" attribute="1" defaultMemberUniqueName="[Ship Date].[Day].[All]" allUniqueName="[Ship Date].[Day].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Full Date]" caption="Ship Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Ship Date].[Full Date].[All]" allUniqueName="[Ship Date].[Full Date].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Month]" caption="Ship Date.Month" attribute="1" defaultMemberUniqueName="[Ship Date].[Month].[All]" allUniqueName="[Ship Date].[Month].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Month Name]" caption="Ship Date.Month Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Month Name].[All]" allUniqueName="[Ship Date].[Month Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Quarter]" caption="Ship Date.Quarter" attribute="1" defaultMemberUniqueName="[Ship Date].[Quarter].[All]" allUniqueName="[Ship Date].[Quarter].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Weekday Name]" caption="Ship Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Weekday Name].[All]" allUniqueName="[Ship Date].[Weekday Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Year]" caption="Ship Date.Year" attribute="1" defaultMemberUniqueName="[Ship Date].[Year].[All]" allUniqueName="[Ship Date].[Year].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Sales]" caption="Sales" measure="1" displayFolder="" measureGroup="Fact Sales" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="6"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Quantity]" caption="Quantity" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Discount]" caption="Discount" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Profit]" caption="Profit" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Delivery Days]" caption="Delivery Days" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Fact Sales Count]" caption="Fact Sales Count" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Profit Margin]" caption="Profit Margin" measure="1" displayFolder="" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Avg Delivery Days]" caption="Avg Delivery Days" measure="1" displayFolder="" count="0"/>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="7">
+    <dimension name="Dim Customer" uniqueName="[Dim Customer]" caption="Dim Customer"/>
+    <dimension name="Dim Geography" uniqueName="[Dim Geography]" caption="Dim Geography"/>
+    <dimension name="Dim Product" uniqueName="[Dim Product]" caption="Dim Product"/>
+    <dimension name="Dim Ship Mode" uniqueName="[Dim Ship Mode]" caption="Dim Ship Mode"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Order Date" uniqueName="[Order Date]" caption="Order Date"/>
+    <dimension name="Ship Date" uniqueName="[Ship Date]" caption="Ship Date"/>
+  </dimensions>
+  <measureGroups count="1">
+    <measureGroup name="Fact Sales" caption="Fact Sales"/>
+  </measureGroups>
+  <maps count="6">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="0" dimension="2"/>
+    <map measureGroup="0" dimension="3"/>
+    <map measureGroup="0" dimension="5"/>
+    <map measureGroup="0" dimension="6"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46206.740128472222" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{15D6C767-A6EA-480E-9AA5-FEB4576400B1}">
+  <cacheSource type="external" connectionId="1"/>
+  <cacheFields count="6">
+    <cacheField name="[Dim Customer].[Customer].[Segment]" caption="Segment" numFmtId="0" level="1">
+      <sharedItems count="3">
+        <s v="[Dim Customer].[Customer].[Segment].&amp;[Consumer]" c="Consumer"/>
+        <s v="[Dim Customer].[Customer].[Segment].&amp;[Corporate]" c="Corporate"/>
+        <s v="[Dim Customer].[Customer].[Segment].&amp;[Home Office]" c="Home Office"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Dim Customer].[Customer].[Customer Name]" caption="Customer Name" numFmtId="0" level="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Dim Customer].[Customer].[Customer Name].[Customer ID]" caption="Customer ID" propertyName="Customer ID" numFmtId="0" level="2" memberPropertyField="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Dim Customer].[Customer].[Customer Name].[Segment]" caption="Segment" propertyName="Segment" numFmtId="0" level="2" memberPropertyField="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[Measures].[Profit]" caption="Profit" numFmtId="0" hierarchy="35" level="32767"/>
+    <cacheField name="[Order Date].[Year].[Year]" caption="Year" numFmtId="0" hierarchy="23" level="1">
+      <sharedItems count="4">
+        <s v="[Order Date].[Year].&amp;[2014]" c="2014"/>
+        <s v="[Order Date].[Year].&amp;[2015]" c="2015"/>
+        <s v="[Order Date].[Year].&amp;[2016]" c="2016"/>
+        <s v="[Order Date].[Year].&amp;[2017]" c="2017"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <cacheHierarchies count="40">
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer]" caption="Customer" defaultMemberUniqueName="[Dim Customer].[Customer].[All]" allUniqueName="[Dim Customer].[Customer].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="3" unbalanced="0">
+      <fieldsUsage count="3">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[Dim Customer].[Customer ID].[All]" allUniqueName="[Dim Customer].[Customer ID].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Customer Name]" caption="Customer Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Customer].[Customer Name].[All]" allUniqueName="[Dim Customer].[Customer Name].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Dim Customer].[Segment].[All]" allUniqueName="[Dim Customer].[Segment].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[City]" caption="City" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Geography].[City].[All]" allUniqueName="[Dim Geography].[City].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Dim Geography].[Country].[All]" allUniqueName="[Dim Geography].[Country].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Geography]" caption="Geography" defaultMemberUniqueName="[Dim Geography].[Geography].[All]" allUniqueName="[Dim Geography].[Geography].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Postal Code]" caption="Postal Code" attribute="1" defaultMemberUniqueName="[Dim Geography].[Postal Code].[All]" allUniqueName="[Dim Geography].[Postal Code].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[Region]" caption="Region" attribute="1" defaultMemberUniqueName="[Dim Geography].[Region].[All]" allUniqueName="[Dim Geography].[Region].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Geography].[State]" caption="State" attribute="1" defaultMemberUniqueName="[Dim Geography].[State].[All]" allUniqueName="[Dim Geography].[State].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Category].[All]" allUniqueName="[Dim Product].[Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product]" caption="Product" defaultMemberUniqueName="[Dim Product].[Product].[All]" allUniqueName="[Dim Product].[Product].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product ID]" caption="Product ID" attribute="1" defaultMemberUniqueName="[Dim Product].[Product ID].[All]" allUniqueName="[Dim Product].[Product ID].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Product Name]" caption="Product Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Product].[Product Name].[All]" allUniqueName="[Dim Product].[Product Name].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Product].[Sub Category]" caption="Sub Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Sub Category].[All]" allUniqueName="[Dim Product].[Sub Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Dim Ship Mode].[Ship Mode]" caption="Ship Mode" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Ship Mode].[Ship Mode].[All]" allUniqueName="[Dim Ship Mode].[Ship Mode].[All]" dimensionUniqueName="[Dim Ship Mode]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Calendar]" caption="Order Date.Calendar" defaultMemberUniqueName="[Order Date].[Calendar].[All]" allUniqueName="[Order Date].[Calendar].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Day]" caption="Order Date.Day" attribute="1" defaultMemberUniqueName="[Order Date].[Day].[All]" allUniqueName="[Order Date].[Day].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Full Date]" caption="Order Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Order Date].[Full Date].[All]" allUniqueName="[Order Date].[Full Date].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Month]" caption="Order Date.Month" attribute="1" defaultMemberUniqueName="[Order Date].[Month].[All]" allUniqueName="[Order Date].[Month].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Month Name]" caption="Order Date.Month Name" attribute="1" defaultMemberUniqueName="[Order Date].[Month Name].[All]" allUniqueName="[Order Date].[Month Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Quarter]" caption="Order Date.Quarter" attribute="1" defaultMemberUniqueName="[Order Date].[Quarter].[All]" allUniqueName="[Order Date].[Quarter].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Weekday Name]" caption="Order Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Order Date].[Weekday Name].[All]" allUniqueName="[Order Date].[Weekday Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Order Date].[Year]" caption="Order Date.Year" attribute="1" defaultMemberUniqueName="[Order Date].[Year].[All]" allUniqueName="[Order Date].[Year].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="2" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="5"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Ship Date].[Calendar]" caption="Ship Date.Calendar" defaultMemberUniqueName="[Ship Date].[Calendar].[All]" allUniqueName="[Ship Date].[Calendar].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Day]" caption="Ship Date.Day" attribute="1" defaultMemberUniqueName="[Ship Date].[Day].[All]" allUniqueName="[Ship Date].[Day].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Full Date]" caption="Ship Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Ship Date].[Full Date].[All]" allUniqueName="[Ship Date].[Full Date].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Month]" caption="Ship Date.Month" attribute="1" defaultMemberUniqueName="[Ship Date].[Month].[All]" allUniqueName="[Ship Date].[Month].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Month Name]" caption="Ship Date.Month Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Month Name].[All]" allUniqueName="[Ship Date].[Month Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Quarter]" caption="Ship Date.Quarter" attribute="1" defaultMemberUniqueName="[Ship Date].[Quarter].[All]" allUniqueName="[Ship Date].[Quarter].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Weekday Name]" caption="Ship Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Weekday Name].[All]" allUniqueName="[Ship Date].[Weekday Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Ship Date].[Year]" caption="Ship Date.Year" attribute="1" defaultMemberUniqueName="[Ship Date].[Year].[All]" allUniqueName="[Ship Date].[Year].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Sales]" caption="Sales" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Quantity]" caption="Quantity" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Discount]" caption="Discount" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Profit]" caption="Profit" measure="1" displayFolder="" measureGroup="Fact Sales" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="4"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Delivery Days]" caption="Delivery Days" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Fact Sales Count]" caption="Fact Sales Count" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Profit Margin]" caption="Profit Margin" measure="1" displayFolder="" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Avg Delivery Days]" caption="Avg Delivery Days" measure="1" displayFolder="" count="0"/>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="7">
+    <dimension name="Dim Customer" uniqueName="[Dim Customer]" caption="Dim Customer"/>
+    <dimension name="Dim Geography" uniqueName="[Dim Geography]" caption="Dim Geography"/>
+    <dimension name="Dim Product" uniqueName="[Dim Product]" caption="Dim Product"/>
+    <dimension name="Dim Ship Mode" uniqueName="[Dim Ship Mode]" caption="Dim Ship Mode"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Order Date" uniqueName="[Order Date]" caption="Order Date"/>
+    <dimension name="Ship Date" uniqueName="[Ship Date]" caption="Ship Date"/>
+  </dimensions>
+  <measureGroups count="1">
+    <measureGroup name="Fact Sales" caption="Fact Sales"/>
+  </measureGroups>
+  <maps count="6">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="0" dimension="2"/>
+    <map measureGroup="0" dimension="3"/>
+    <map measureGroup="0" dimension="5"/>
+    <map measureGroup="0" dimension="6"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46206.740129050922" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{16152C29-77A8-44C6-B6A6-9557FF558682}">
   <cacheSource type="external" connectionId="1"/>
   <cacheFields count="11">
     <cacheField name="[Measures].[Sales]" caption="Sales" numFmtId="0" hierarchy="32" level="32767"/>
@@ -5128,340 +5460,8 @@
 </pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46181.646090046299" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{15D6C767-A6EA-480E-9AA5-FEB4576400B1}">
-  <cacheSource type="external" connectionId="1"/>
-  <cacheFields count="6">
-    <cacheField name="[Dim Customer].[Customer].[Segment]" caption="Segment" numFmtId="0" level="1">
-      <sharedItems count="3">
-        <s v="[Dim Customer].[Customer].[Segment].&amp;[Consumer]" c="Consumer"/>
-        <s v="[Dim Customer].[Customer].[Segment].&amp;[Corporate]" c="Corporate"/>
-        <s v="[Dim Customer].[Customer].[Segment].&amp;[Home Office]" c="Home Office"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Dim Customer].[Customer].[Customer Name]" caption="Customer Name" numFmtId="0" level="2">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Dim Customer].[Customer].[Customer Name].[Customer ID]" caption="Customer ID" propertyName="Customer ID" numFmtId="0" level="2" memberPropertyField="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Dim Customer].[Customer].[Customer Name].[Segment]" caption="Segment" propertyName="Segment" numFmtId="0" level="2" memberPropertyField="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Measures].[Profit]" caption="Profit" numFmtId="0" hierarchy="35" level="32767"/>
-    <cacheField name="[Order Date].[Year].[Year]" caption="Year" numFmtId="0" hierarchy="23" level="1">
-      <sharedItems count="4">
-        <s v="[Order Date].[Year].&amp;[2014]" c="2014"/>
-        <s v="[Order Date].[Year].&amp;[2015]" c="2015"/>
-        <s v="[Order Date].[Year].&amp;[2016]" c="2016"/>
-        <s v="[Order Date].[Year].&amp;[2017]" c="2017"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="40">
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer]" caption="Customer" defaultMemberUniqueName="[Dim Customer].[Customer].[All]" allUniqueName="[Dim Customer].[Customer].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="3" unbalanced="0">
-      <fieldsUsage count="3">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[Dim Customer].[Customer ID].[All]" allUniqueName="[Dim Customer].[Customer ID].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer Name]" caption="Customer Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Customer].[Customer Name].[All]" allUniqueName="[Dim Customer].[Customer Name].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Dim Customer].[Segment].[All]" allUniqueName="[Dim Customer].[Segment].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[City]" caption="City" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Geography].[City].[All]" allUniqueName="[Dim Geography].[City].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Dim Geography].[Country].[All]" allUniqueName="[Dim Geography].[Country].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Geography]" caption="Geography" defaultMemberUniqueName="[Dim Geography].[Geography].[All]" allUniqueName="[Dim Geography].[Geography].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Postal Code]" caption="Postal Code" attribute="1" defaultMemberUniqueName="[Dim Geography].[Postal Code].[All]" allUniqueName="[Dim Geography].[Postal Code].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Region]" caption="Region" attribute="1" defaultMemberUniqueName="[Dim Geography].[Region].[All]" allUniqueName="[Dim Geography].[Region].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[State]" caption="State" attribute="1" defaultMemberUniqueName="[Dim Geography].[State].[All]" allUniqueName="[Dim Geography].[State].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Category].[All]" allUniqueName="[Dim Product].[Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product]" caption="Product" defaultMemberUniqueName="[Dim Product].[Product].[All]" allUniqueName="[Dim Product].[Product].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product ID]" caption="Product ID" attribute="1" defaultMemberUniqueName="[Dim Product].[Product ID].[All]" allUniqueName="[Dim Product].[Product ID].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product Name]" caption="Product Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Product].[Product Name].[All]" allUniqueName="[Dim Product].[Product Name].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Sub Category]" caption="Sub Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Sub Category].[All]" allUniqueName="[Dim Product].[Sub Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Ship Mode].[Ship Mode]" caption="Ship Mode" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Ship Mode].[Ship Mode].[All]" allUniqueName="[Dim Ship Mode].[Ship Mode].[All]" dimensionUniqueName="[Dim Ship Mode]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Calendar]" caption="Order Date.Calendar" defaultMemberUniqueName="[Order Date].[Calendar].[All]" allUniqueName="[Order Date].[Calendar].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Day]" caption="Order Date.Day" attribute="1" defaultMemberUniqueName="[Order Date].[Day].[All]" allUniqueName="[Order Date].[Day].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Full Date]" caption="Order Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Order Date].[Full Date].[All]" allUniqueName="[Order Date].[Full Date].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Month]" caption="Order Date.Month" attribute="1" defaultMemberUniqueName="[Order Date].[Month].[All]" allUniqueName="[Order Date].[Month].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Month Name]" caption="Order Date.Month Name" attribute="1" defaultMemberUniqueName="[Order Date].[Month Name].[All]" allUniqueName="[Order Date].[Month Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Quarter]" caption="Order Date.Quarter" attribute="1" defaultMemberUniqueName="[Order Date].[Quarter].[All]" allUniqueName="[Order Date].[Quarter].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Weekday Name]" caption="Order Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Order Date].[Weekday Name].[All]" allUniqueName="[Order Date].[Weekday Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Year]" caption="Order Date.Year" attribute="1" defaultMemberUniqueName="[Order Date].[Year].[All]" allUniqueName="[Order Date].[Year].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="2" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="5"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Ship Date].[Calendar]" caption="Ship Date.Calendar" defaultMemberUniqueName="[Ship Date].[Calendar].[All]" allUniqueName="[Ship Date].[Calendar].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Day]" caption="Ship Date.Day" attribute="1" defaultMemberUniqueName="[Ship Date].[Day].[All]" allUniqueName="[Ship Date].[Day].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Full Date]" caption="Ship Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Ship Date].[Full Date].[All]" allUniqueName="[Ship Date].[Full Date].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Month]" caption="Ship Date.Month" attribute="1" defaultMemberUniqueName="[Ship Date].[Month].[All]" allUniqueName="[Ship Date].[Month].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Month Name]" caption="Ship Date.Month Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Month Name].[All]" allUniqueName="[Ship Date].[Month Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Quarter]" caption="Ship Date.Quarter" attribute="1" defaultMemberUniqueName="[Ship Date].[Quarter].[All]" allUniqueName="[Ship Date].[Quarter].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Weekday Name]" caption="Ship Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Weekday Name].[All]" allUniqueName="[Ship Date].[Weekday Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Year]" caption="Ship Date.Year" attribute="1" defaultMemberUniqueName="[Ship Date].[Year].[All]" allUniqueName="[Ship Date].[Year].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Sales]" caption="Sales" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Quantity]" caption="Quantity" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Discount]" caption="Discount" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Profit]" caption="Profit" measure="1" displayFolder="" measureGroup="Fact Sales" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="4"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Delivery Days]" caption="Delivery Days" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Fact Sales Count]" caption="Fact Sales Count" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Profit Margin]" caption="Profit Margin" measure="1" displayFolder="" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Avg Delivery Days]" caption="Avg Delivery Days" measure="1" displayFolder="" count="0"/>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="7">
-    <dimension name="Dim Customer" uniqueName="[Dim Customer]" caption="Dim Customer"/>
-    <dimension name="Dim Geography" uniqueName="[Dim Geography]" caption="Dim Geography"/>
-    <dimension name="Dim Product" uniqueName="[Dim Product]" caption="Dim Product"/>
-    <dimension name="Dim Ship Mode" uniqueName="[Dim Ship Mode]" caption="Dim Ship Mode"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Order Date" uniqueName="[Order Date]" caption="Order Date"/>
-    <dimension name="Ship Date" uniqueName="[Ship Date]" caption="Ship Date"/>
-  </dimensions>
-  <measureGroups count="1">
-    <measureGroup name="Fact Sales" caption="Fact Sales"/>
-  </measureGroups>
-  <maps count="6">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="0" dimension="2"/>
-    <map measureGroup="0" dimension="3"/>
-    <map measureGroup="0" dimension="5"/>
-    <map measureGroup="0" dimension="6"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46181.646093055555" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{2B00A886-4FF8-4527-B1CA-9D438D508401}">
-  <cacheSource type="external" connectionId="1"/>
-  <cacheFields count="8">
-    <cacheField name="[Dim Product].[Product].[Category]" caption="Category" numFmtId="0" hierarchy="11" level="1">
-      <sharedItems count="3">
-        <s v="[Dim Product].[Product].[Category].&amp;[Furniture]" c="Furniture"/>
-        <s v="[Dim Product].[Product].[Category].&amp;[Office Supplies]" c="Office Supplies"/>
-        <s v="[Dim Product].[Product].[Category].&amp;[Technology]" c="Technology"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Dim Product].[Product].[Sub Category]" caption="Sub Category" numFmtId="0" hierarchy="11" level="2">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Dim Product].[Product].[Product Name]" caption="Product Name" numFmtId="0" hierarchy="11" level="3">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Dim Product].[Product].[Product Name].[Category]" caption="Category" propertyName="Category" numFmtId="0" hierarchy="11" level="3" memberPropertyField="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Dim Product].[Product].[Product Name].[Product ID]" caption="Product ID" propertyName="Product ID" numFmtId="0" hierarchy="11" level="3" memberPropertyField="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Dim Product].[Product].[Product Name].[Sub Category]" caption="Sub Category" propertyName="Sub Category" numFmtId="0" hierarchy="11" level="3" memberPropertyField="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[Measures].[Sales]" caption="Sales" numFmtId="0" hierarchy="32" level="32767"/>
-    <cacheField name="[Dim Geography].[Region].[Region]" caption="Region" numFmtId="0" hierarchy="8" level="1">
-      <sharedItems count="4">
-        <s v="[Dim Geography].[Region].&amp;[Central]" c="Central"/>
-        <s v="[Dim Geography].[Region].&amp;[East]" c="East"/>
-        <s v="[Dim Geography].[Region].&amp;[South]" c="South"/>
-        <s v="[Dim Geography].[Region].&amp;[West]" c="West"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="40">
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer]" caption="Customer" defaultMemberUniqueName="[Dim Customer].[Customer].[All]" allUniqueName="[Dim Customer].[Customer].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[Dim Customer].[Customer ID].[All]" allUniqueName="[Dim Customer].[Customer ID].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer Name]" caption="Customer Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Customer].[Customer Name].[All]" allUniqueName="[Dim Customer].[Customer Name].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Dim Customer].[Segment].[All]" allUniqueName="[Dim Customer].[Segment].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[City]" caption="City" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Geography].[City].[All]" allUniqueName="[Dim Geography].[City].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Dim Geography].[Country].[All]" allUniqueName="[Dim Geography].[Country].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Geography]" caption="Geography" defaultMemberUniqueName="[Dim Geography].[Geography].[All]" allUniqueName="[Dim Geography].[Geography].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Postal Code]" caption="Postal Code" attribute="1" defaultMemberUniqueName="[Dim Geography].[Postal Code].[All]" allUniqueName="[Dim Geography].[Postal Code].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Region]" caption="Region" attribute="1" defaultMemberUniqueName="[Dim Geography].[Region].[All]" allUniqueName="[Dim Geography].[Region].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="2" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="7"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Dim Geography].[State]" caption="State" attribute="1" defaultMemberUniqueName="[Dim Geography].[State].[All]" allUniqueName="[Dim Geography].[State].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Category].[All]" allUniqueName="[Dim Product].[Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product]" caption="Product" defaultMemberUniqueName="[Dim Product].[Product].[All]" allUniqueName="[Dim Product].[Product].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="4" unbalanced="0">
-      <fieldsUsage count="4">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-        <fieldUsage x="1"/>
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Dim Product].[Product ID]" caption="Product ID" attribute="1" defaultMemberUniqueName="[Dim Product].[Product ID].[All]" allUniqueName="[Dim Product].[Product ID].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product Name]" caption="Product Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Product].[Product Name].[All]" allUniqueName="[Dim Product].[Product Name].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Sub Category]" caption="Sub Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Sub Category].[All]" allUniqueName="[Dim Product].[Sub Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Ship Mode].[Ship Mode]" caption="Ship Mode" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Ship Mode].[Ship Mode].[All]" allUniqueName="[Dim Ship Mode].[Ship Mode].[All]" dimensionUniqueName="[Dim Ship Mode]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Calendar]" caption="Order Date.Calendar" defaultMemberUniqueName="[Order Date].[Calendar].[All]" allUniqueName="[Order Date].[Calendar].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Day]" caption="Order Date.Day" attribute="1" defaultMemberUniqueName="[Order Date].[Day].[All]" allUniqueName="[Order Date].[Day].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Full Date]" caption="Order Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Order Date].[Full Date].[All]" allUniqueName="[Order Date].[Full Date].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Month]" caption="Order Date.Month" attribute="1" defaultMemberUniqueName="[Order Date].[Month].[All]" allUniqueName="[Order Date].[Month].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Month Name]" caption="Order Date.Month Name" attribute="1" defaultMemberUniqueName="[Order Date].[Month Name].[All]" allUniqueName="[Order Date].[Month Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Quarter]" caption="Order Date.Quarter" attribute="1" defaultMemberUniqueName="[Order Date].[Quarter].[All]" allUniqueName="[Order Date].[Quarter].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Weekday Name]" caption="Order Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Order Date].[Weekday Name].[All]" allUniqueName="[Order Date].[Weekday Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Year]" caption="Order Date.Year" attribute="1" defaultMemberUniqueName="[Order Date].[Year].[All]" allUniqueName="[Order Date].[Year].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Calendar]" caption="Ship Date.Calendar" defaultMemberUniqueName="[Ship Date].[Calendar].[All]" allUniqueName="[Ship Date].[Calendar].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Day]" caption="Ship Date.Day" attribute="1" defaultMemberUniqueName="[Ship Date].[Day].[All]" allUniqueName="[Ship Date].[Day].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Full Date]" caption="Ship Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Ship Date].[Full Date].[All]" allUniqueName="[Ship Date].[Full Date].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Month]" caption="Ship Date.Month" attribute="1" defaultMemberUniqueName="[Ship Date].[Month].[All]" allUniqueName="[Ship Date].[Month].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Month Name]" caption="Ship Date.Month Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Month Name].[All]" allUniqueName="[Ship Date].[Month Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Quarter]" caption="Ship Date.Quarter" attribute="1" defaultMemberUniqueName="[Ship Date].[Quarter].[All]" allUniqueName="[Ship Date].[Quarter].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Weekday Name]" caption="Ship Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Weekday Name].[All]" allUniqueName="[Ship Date].[Weekday Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Year]" caption="Ship Date.Year" attribute="1" defaultMemberUniqueName="[Ship Date].[Year].[All]" allUniqueName="[Ship Date].[Year].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Sales]" caption="Sales" measure="1" displayFolder="" measureGroup="Fact Sales" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="6"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Quantity]" caption="Quantity" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Discount]" caption="Discount" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Profit]" caption="Profit" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Delivery Days]" caption="Delivery Days" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Fact Sales Count]" caption="Fact Sales Count" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Profit Margin]" caption="Profit Margin" measure="1" displayFolder="" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Avg Delivery Days]" caption="Avg Delivery Days" measure="1" displayFolder="" count="0"/>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="7">
-    <dimension name="Dim Customer" uniqueName="[Dim Customer]" caption="Dim Customer"/>
-    <dimension name="Dim Geography" uniqueName="[Dim Geography]" caption="Dim Geography"/>
-    <dimension name="Dim Product" uniqueName="[Dim Product]" caption="Dim Product"/>
-    <dimension name="Dim Ship Mode" uniqueName="[Dim Ship Mode]" caption="Dim Ship Mode"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Order Date" uniqueName="[Order Date]" caption="Order Date"/>
-    <dimension name="Ship Date" uniqueName="[Ship Date]" caption="Ship Date"/>
-  </dimensions>
-  <measureGroups count="1">
-    <measureGroup name="Fact Sales" caption="Fact Sales"/>
-  </measureGroups>
-  <maps count="6">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="0" dimension="2"/>
-    <map measureGroup="0" dimension="3"/>
-    <map measureGroup="0" dimension="5"/>
-    <map measureGroup="0" dimension="6"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="MY MSI" refreshedDate="46183.571962615744" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{8648899E-E912-41E9-AC6C-35175A7D3FBA}">
-  <cacheSource type="external" connectionId="2"/>
-  <cacheFields count="2">
-    <cacheField name="[Dim Product].[Category].[Category]" caption="Category" numFmtId="0" hierarchy="10" level="1">
-      <sharedItems count="3">
-        <s v="[Dim Product].[Category].&amp;[Furniture]" c="Furniture"/>
-        <s v="[Dim Product].[Category].&amp;[Office Supplies]" c="Office Supplies"/>
-        <s v="[Dim Product].[Category].&amp;[Technology]" c="Technology"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Measures].[Profit Margin]" caption="Profit Margin" numFmtId="0" hierarchy="38" level="32767"/>
-  </cacheFields>
-  <cacheHierarchies count="40">
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer]" caption="Customer" defaultMemberUniqueName="[Dim Customer].[Customer].[All]" allUniqueName="[Dim Customer].[Customer].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="3" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[Dim Customer].[Customer ID].[All]" allUniqueName="[Dim Customer].[Customer ID].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Customer Name]" caption="Customer Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Customer].[Customer Name].[All]" allUniqueName="[Dim Customer].[Customer Name].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Dim Customer].[Segment].[All]" allUniqueName="[Dim Customer].[Segment].[All]" dimensionUniqueName="[Dim Customer]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[City]" caption="City" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Geography].[City].[All]" allUniqueName="[Dim Geography].[City].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Dim Geography].[Country].[All]" allUniqueName="[Dim Geography].[Country].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Geography]" caption="Geography" defaultMemberUniqueName="[Dim Geography].[Geography].[All]" allUniqueName="[Dim Geography].[Geography].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Postal Code]" caption="Postal Code" attribute="1" defaultMemberUniqueName="[Dim Geography].[Postal Code].[All]" allUniqueName="[Dim Geography].[Postal Code].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[Region]" caption="Region" attribute="1" defaultMemberUniqueName="[Dim Geography].[Region].[All]" allUniqueName="[Dim Geography].[Region].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Geography].[State]" caption="State" attribute="1" defaultMemberUniqueName="[Dim Geography].[State].[All]" allUniqueName="[Dim Geography].[State].[All]" dimensionUniqueName="[Dim Geography]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Category].[All]" allUniqueName="[Dim Product].[Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="2" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Dim Product].[Product]" caption="Product" defaultMemberUniqueName="[Dim Product].[Product].[All]" allUniqueName="[Dim Product].[Product].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="4" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product ID]" caption="Product ID" attribute="1" defaultMemberUniqueName="[Dim Product].[Product ID].[All]" allUniqueName="[Dim Product].[Product ID].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Product Name]" caption="Product Name" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Product].[Product Name].[All]" allUniqueName="[Dim Product].[Product Name].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Product].[Sub Category]" caption="Sub Category" attribute="1" defaultMemberUniqueName="[Dim Product].[Sub Category].[All]" allUniqueName="[Dim Product].[Sub Category].[All]" dimensionUniqueName="[Dim Product]" displayFolder="" count="2" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Dim Ship Mode].[Ship Mode]" caption="Ship Mode" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Dim Ship Mode].[Ship Mode].[All]" allUniqueName="[Dim Ship Mode].[Ship Mode].[All]" dimensionUniqueName="[Dim Ship Mode]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Calendar]" caption="Order Date.Calendar" defaultMemberUniqueName="[Order Date].[Calendar].[All]" allUniqueName="[Order Date].[Calendar].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Day]" caption="Order Date.Day" attribute="1" defaultMemberUniqueName="[Order Date].[Day].[All]" allUniqueName="[Order Date].[Day].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Full Date]" caption="Order Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Order Date].[Full Date].[All]" allUniqueName="[Order Date].[Full Date].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Month]" caption="Order Date.Month" attribute="1" defaultMemberUniqueName="[Order Date].[Month].[All]" allUniqueName="[Order Date].[Month].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Month Name]" caption="Order Date.Month Name" attribute="1" defaultMemberUniqueName="[Order Date].[Month Name].[All]" allUniqueName="[Order Date].[Month Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Quarter]" caption="Order Date.Quarter" attribute="1" defaultMemberUniqueName="[Order Date].[Quarter].[All]" allUniqueName="[Order Date].[Quarter].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Weekday Name]" caption="Order Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Order Date].[Weekday Name].[All]" allUniqueName="[Order Date].[Weekday Name].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Order Date].[Year]" caption="Order Date.Year" attribute="1" defaultMemberUniqueName="[Order Date].[Year].[All]" allUniqueName="[Order Date].[Year].[All]" dimensionUniqueName="[Order Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Calendar]" caption="Ship Date.Calendar" defaultMemberUniqueName="[Ship Date].[Calendar].[All]" allUniqueName="[Ship Date].[Calendar].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Day]" caption="Ship Date.Day" attribute="1" defaultMemberUniqueName="[Ship Date].[Day].[All]" allUniqueName="[Ship Date].[Day].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Full Date]" caption="Ship Date.Full Date" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Ship Date].[Full Date].[All]" allUniqueName="[Ship Date].[Full Date].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Month]" caption="Ship Date.Month" attribute="1" defaultMemberUniqueName="[Ship Date].[Month].[All]" allUniqueName="[Ship Date].[Month].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Month Name]" caption="Ship Date.Month Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Month Name].[All]" allUniqueName="[Ship Date].[Month Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Quarter]" caption="Ship Date.Quarter" attribute="1" defaultMemberUniqueName="[Ship Date].[Quarter].[All]" allUniqueName="[Ship Date].[Quarter].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Weekday Name]" caption="Ship Date.Weekday Name" attribute="1" defaultMemberUniqueName="[Ship Date].[Weekday Name].[All]" allUniqueName="[Ship Date].[Weekday Name].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Ship Date].[Year]" caption="Ship Date.Year" attribute="1" defaultMemberUniqueName="[Ship Date].[Year].[All]" allUniqueName="[Ship Date].[Year].[All]" dimensionUniqueName="[Ship Date]" displayFolder="" count="0" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Sales]" caption="Sales" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Quantity]" caption="Quantity" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Discount]" caption="Discount" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Profit]" caption="Profit" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Delivery Days]" caption="Delivery Days" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Fact Sales Count]" caption="Fact Sales Count" measure="1" displayFolder="" measureGroup="Fact Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Profit Margin]" caption="Profit Margin" measure="1" displayFolder="" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Avg Delivery Days]" caption="Avg Delivery Days" measure="1" displayFolder="" count="0"/>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="7">
-    <dimension name="Dim Customer" uniqueName="[Dim Customer]" caption="Dim Customer"/>
-    <dimension name="Dim Geography" uniqueName="[Dim Geography]" caption="Dim Geography"/>
-    <dimension name="Dim Product" uniqueName="[Dim Product]" caption="Dim Product"/>
-    <dimension name="Dim Ship Mode" uniqueName="[Dim Ship Mode]" caption="Dim Ship Mode"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Order Date" uniqueName="[Order Date]" caption="Order Date"/>
-    <dimension name="Ship Date" uniqueName="[Ship Date]" caption="Ship Date"/>
-  </dimensions>
-  <measureGroups count="1">
-    <measureGroup name="Fact Sales" caption="Fact Sales"/>
-  </measureGroups>
-  <maps count="6">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="0" dimension="2"/>
-    <map measureGroup="0" dimension="3"/>
-    <map measureGroup="0" dimension="5"/>
-    <map measureGroup="0" dimension="6"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4893D13-FCFD-4BAE-87CD-BCABB8FA824C}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4893D13-FCFD-4BAE-87CD-BCABB8FA824C}" name="PivotTable1" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" fieldListSortAscending="1">
   <location ref="A3:F8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0">
@@ -5688,7 +5688,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C09D1A3D-59E8-4676-A76A-6090323E52E3}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C09D1A3D-59E8-4676-A76A-6090323E52E3}" name="PivotTable1" cacheId="36" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A3:F8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0">
@@ -5912,7 +5912,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79B76F23-D2A1-4862-A674-420895809182}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79B76F23-D2A1-4862-A674-420895809182}" name="PivotTable1" cacheId="39" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" fieldListSortAscending="1">
   <location ref="A3:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -6123,7 +6123,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{68F78C19-B0A3-4297-B772-4AD903F468B9}" name="PivotTable1" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{68F78C19-B0A3-4297-B772-4AD903F468B9}" name="PivotTable1" cacheId="30" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -6597,7 +6597,7 @@
         <v>252612.7435000003</v>
       </c>
       <c r="F5" s="3">
-        <v>741999.79530000058</v>
+        <v>741999.79529999977</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -6617,7 +6617,7 @@
         <v>220853.24900000007</v>
       </c>
       <c r="F6" s="3">
-        <v>719047.03200000024</v>
+        <v>719047.0320000028</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -6637,7 +6637,7 @@
         <v>251991.83199999991</v>
       </c>
       <c r="F7" s="3">
-        <v>836154.03300000005</v>
+        <v>836154.03299999656</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -6657,7 +6657,7 @@
         <v>725457.82450000034</v>
       </c>
       <c r="F8" s="3">
-        <v>2297200.8602999966</v>
+        <v>2297200.8602999989</v>
       </c>
     </row>
   </sheetData>
@@ -6786,7 +6786,7 @@
         <v>93439.2696</v>
       </c>
       <c r="F8" s="3">
-        <v>286397.02170000016</v>
+        <v>286397.02169999998</v>
       </c>
     </row>
   </sheetData>
@@ -6958,7 +6958,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="4">
-        <v>0.12467217240315598</v>
+        <v>0.1246721724031561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>